<commit_message>
Add LEAPS scanner, voice tool, and new valuations
- New LEAPS finder pipeline (tools/leaps_scanner.py, config/leaps_universe.yaml)
- New voice tool (tools/voice.py) and orchestrator updates
- New valuations: CNR, CNR_TO, DLG_MI, DUOL, NEM, NEM_DE, RMS_PA, SMG_SW, SOIL_TO, SPOT, SU_TO, UBER, 000660_KS
- Updated theses: HIMS, MC_PA, TSLA, WCP_TO with thesis_data.json + history
- Dashboard, scheduler, telegram_bot, screener_engine, thesis_reviewer improvements
- Remove obsolete thesis_rewrite_tracker.md (28/34 pre-rewrite tracking)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/valuations/HIMS/HIMS_modelo_valoracion.xlsx
+++ b/data/valuations/HIMS/HIMS_modelo_valoracion.xlsx
@@ -638,19 +638,19 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.284</v>
+        <v>0.18</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.2556</v>
+        <v>0.15</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.2272</v>
+        <v>0.13</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>0.1988</v>
+        <v>0.1</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.1704</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="9">
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.3692</v>
+        <v>0.22</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.33228</v>
+        <v>0.2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0.29536</v>
+        <v>0.18</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>0.2584399999999999</v>
+        <v>0.14</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.22152</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
@@ -682,19 +682,19 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.1988</v>
+        <v>0.1</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.17892</v>
+        <v>0.08</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>0.15904</v>
+        <v>0.05</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0.13916</v>
+        <v>0.04</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0.11928</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="11">
@@ -775,19 +775,19 @@
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0.7821157918099402</v>
+        <v>0.78</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.7821157918099402</v>
+        <v>0.78</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>0.7821157918099402</v>
+        <v>0.78</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.7821157918099402</v>
+        <v>0.78</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0.7821157918099402</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="16">
@@ -797,19 +797,19 @@
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.8021157918099402</v>
+        <v>0.79</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.8021157918099402</v>
+        <v>0.79</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.8021157918099402</v>
+        <v>0.79</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>0.8021157918099402</v>
+        <v>0.79</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0.8021157918099402</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="17">
@@ -819,19 +819,19 @@
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0.7621157918099402</v>
+        <v>0.76</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.7621157918099402</v>
+        <v>0.76</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>0.7621157918099402</v>
+        <v>0.76</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>0.7621157918099402</v>
+        <v>0.76</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0.7621157918099402</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="18">
@@ -868,19 +868,19 @@
         </is>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.6114327231058824</v>
+        <v>0.55</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.6114327231058824</v>
+        <v>0.55</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.6114327231058824</v>
+        <v>0.55</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>0.6114327231058824</v>
+        <v>0.55</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0.6114327231058824</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="21">
@@ -890,19 +890,19 @@
         </is>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0.6014327231058824</v>
+        <v>0.52</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.6014327231058824</v>
+        <v>0.52</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.6014327231058824</v>
+        <v>0.52</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0.6014327231058824</v>
+        <v>0.52</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0.6014327231058824</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="22">
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0.6214327231058824</v>
+        <v>0.58</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.6214327231058824</v>
+        <v>0.58</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.6214327231058824</v>
+        <v>0.58</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.6214327231058824</v>
+        <v>0.58</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>0.6214327231058824</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="23">
@@ -961,19 +961,19 @@
         </is>
       </c>
       <c r="G25" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="K25" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="26">
@@ -983,19 +983,19 @@
         </is>
       </c>
       <c r="G26" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>0.05694283017111235</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="27">
@@ -1005,19 +1005,19 @@
         </is>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0.06194283017111234</v>
+        <v>0.05</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0.06194283017111234</v>
+        <v>0.05</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>0.06194283017111234</v>
+        <v>0.05</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.06194283017111234</v>
+        <v>0.05</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>0.06194283017111234</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="28">
@@ -1054,19 +1054,19 @@
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>0.01497125285114198</v>
+        <v>0.015</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.01497125285114198</v>
+        <v>0.015</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>0.01497125285114198</v>
+        <v>0.015</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.01497125285114198</v>
+        <v>0.015</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>0.01497125285114198</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="31">
@@ -1076,19 +1076,19 @@
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>0.04579862726111469</v>
+        <v>0.03</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.04579862726111469</v>
+        <v>0.03</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>0.04579862726111469</v>
+        <v>0.03</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.04579862726111469</v>
+        <v>0.03</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>0.04579862726111469</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="32">
@@ -1098,19 +1098,19 @@
         </is>
       </c>
       <c r="G32" s="6" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="34">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>0.153</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="36">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>0.143</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="37">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>0.173</v>
+        <v>0.115</v>
       </c>
     </row>
     <row r="38">
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="C40" s="9" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="C42" s="9" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="F2" s="16" t="n">
-        <v>15.74</v>
+        <v>30.56</v>
       </c>
     </row>
     <row r="4">
@@ -3584,7 +3584,7 @@
         </is>
       </c>
       <c r="K21" s="8">
-        <f>K12*$C$16</f>
+        <f>K8*$C$16</f>
         <v/>
       </c>
     </row>
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="C34" s="20">
-        <f>C33/15.74-1</f>
+        <f>C33/30.56-1</f>
         <v/>
       </c>
     </row>
@@ -3727,202 +3727,202 @@
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
+          <t>8x</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>12x</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
           <t>14x</t>
         </is>
       </c>
-      <c r="D38" s="1" t="inlineStr">
+      <c r="G38" s="1" t="inlineStr">
         <is>
           <t>16x</t>
-        </is>
-      </c>
-      <c r="E38" s="1" t="inlineStr">
-        <is>
-          <t>18x</t>
-        </is>
-      </c>
-      <c r="F38" s="1" t="inlineStr">
-        <is>
-          <t>20x</t>
-        </is>
-      </c>
-      <c r="G38" s="1" t="inlineStr">
-        <is>
-          <t>22x</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="21" t="n">
-        <v>0.123</v>
+        <v>0.08</v>
       </c>
       <c r="C39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*14/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*8/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*16/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*10/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*18/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*12/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*20/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*14/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G39" s="22">
-        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$12*22/(1+$A$39)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$39)^1+H$12/(1+$A$39)^2+I$12/(1+$A$39)^3+J$12/(1+$A$39)^4+K$12/(1+$A$39)^5+K$8*16/(1+$A$39)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
-        <v>0.133</v>
+        <v>0.09</v>
       </c>
       <c r="C40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*14/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*8/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*16/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*10/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*18/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*12/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*20/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*14/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G40" s="22">
-        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$12*22/(1+$A$40)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$40)^1+H$12/(1+$A$40)^2+I$12/(1+$A$40)^3+J$12/(1+$A$40)^4+K$12/(1+$A$40)^5+K$8*16/(1+$A$40)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
-        <v>0.143</v>
+        <v>0.1</v>
       </c>
       <c r="C41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*14/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*8/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*16/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*10/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*18/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*12/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*20/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*14/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G41" s="22">
-        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$12*22/(1+$A$41)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$41)^1+H$12/(1+$A$41)^2+I$12/(1+$A$41)^3+J$12/(1+$A$41)^4+K$12/(1+$A$41)^5+K$8*16/(1+$A$41)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="n">
-        <v>0.153</v>
+        <v>0.11</v>
       </c>
       <c r="C42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*14/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*8/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*16/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*10/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E42" s="23">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*18/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*12/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*20/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*14/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G42" s="22">
-        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$12*22/(1+$A$42)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$42)^1+H$12/(1+$A$42)^2+I$12/(1+$A$42)^3+J$12/(1+$A$42)^4+K$12/(1+$A$42)^5+K$8*16/(1+$A$42)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="n">
-        <v>0.163</v>
+        <v>0.12</v>
       </c>
       <c r="C43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*14/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*8/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*16/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*10/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*18/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*12/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*20/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*14/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G43" s="22">
-        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$12*22/(1+$A$43)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$43)^1+H$12/(1+$A$43)^2+I$12/(1+$A$43)^3+J$12/(1+$A$43)^4+K$12/(1+$A$43)^5+K$8*16/(1+$A$43)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="n">
-        <v>0.173</v>
+        <v>0.13</v>
       </c>
       <c r="C44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*14/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*8/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*16/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*10/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*18/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*12/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*20/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*14/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G44" s="22">
-        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$12*22/(1+$A$44)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$44)^1+H$12/(1+$A$44)^2+I$12/(1+$A$44)^3+J$12/(1+$A$44)^4+K$12/(1+$A$44)^5+K$8*16/(1+$A$44)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="n">
-        <v>0.183</v>
+        <v>0.14</v>
       </c>
       <c r="C45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*14/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*8/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="D45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*16/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*10/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="E45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*18/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*12/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="F45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*20/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*14/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
       <c r="G45" s="22">
-        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$12*22/(1+$A$45)^5+$C$29)/$C$32</f>
+        <f>(G$12/(1+$A$45)^1+H$12/(1+$A$45)^2+I$12/(1+$A$45)^3+J$12/(1+$A$45)^4+K$12/(1+$A$45)^5+K$8*16/(1+$A$45)^5+$C$29)/$C$32</f>
         <v/>
       </c>
     </row>

</xml_diff>